<commit_message>
process: Re-extract 141 batch files with improved specs extraction
</commit_message>
<xml_diff>
--- a/output/processing/072-073_S418.xlsx
+++ b/output/processing/072-073_S418.xlsx
@@ -531,19 +531,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="31" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
@@ -649,9 +649,71 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bassO</t>
+          <t>S418 24V</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>220-240V~ 50/60 Hz</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Con spazzole 24V</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>35 W</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>6 Kg</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>823 x 104 x 137 mm</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>IP54</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-20°C ÷ + 55°C</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Uso continuo</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>37 mm/s (con E124)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>350 mm (390 mm senza arresti)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Non compresa</t>
         </is>
       </c>
     </row>

</xml_diff>